<commit_message>
Reclassify BIPO to Corporate Financial Function (week-ending-2026-06-19)
</commit_message>
<xml_diff>
--- a/Weekly_Fintech_Deals_2026-06-19.xlsx
+++ b/Weekly_Fintech_Deals_2026-06-19.xlsx
@@ -894,12 +894,12 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Financial Info &amp; Analytics</t>
+          <t>Corporate Financial Function</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Singapore</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -909,23 +909,23 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Behavox</t>
+          <t>BIPO</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>HPS Investment Partners</t>
+          <t>Apis Partners</t>
         </is>
       </c>
       <c r="F4" s="2" t="n">
-        <v>175</v>
+        <v>50</v>
       </c>
       <c r="G4" s="2" t="inlineStr"/>
       <c r="H4" s="2" t="inlineStr"/>
       <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>AI-native compliance and risk platform that unifies communications surveillance and controls for banks, asset managers, and other regulated institutions</t>
+          <t>Payroll-payments and embedded workforce-finance platform offering global payroll, HR management, and employer-of-record services across 170+ markets</t>
         </is>
       </c>
       <c r="K4" s="3" t="inlineStr">
@@ -937,7 +937,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>InsurTech</t>
+          <t>Financial Info &amp; Analytics</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -947,28 +947,28 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>18-Jun-26</t>
+          <t>17-Jun-26</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Connie Health</t>
+          <t>Behavox</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>HealthQuest Capital</t>
+          <t>HPS Investment Partners</t>
         </is>
       </c>
       <c r="F5" s="2" t="n">
-        <v>40</v>
+        <v>175</v>
       </c>
       <c r="G5" s="2" t="inlineStr"/>
       <c r="H5" s="2" t="inlineStr"/>
       <c r="I5" s="2" t="inlineStr"/>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>AI-native Medicare navigation platform pairing licensed advisors with software to help seniors choose and manage Medicare plans</t>
+          <t>AI-native compliance and risk platform that unifies communications surveillance and controls for banks, asset managers, and other regulated institutions</t>
         </is>
       </c>
       <c r="K5" s="3" t="inlineStr">
@@ -980,7 +980,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Payments</t>
+          <t>InsurTech</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -990,28 +990,28 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>16-Jun-26</t>
+          <t>18-Jun-26</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Flutterwave</t>
+          <t>Connie Health</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Ripple (strategic)</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr"/>
-      <c r="G6" s="2" t="n">
-        <v>3200</v>
-      </c>
+          <t>HealthQuest Capital</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="G6" s="2" t="inlineStr"/>
       <c r="H6" s="2" t="inlineStr"/>
       <c r="I6" s="2" t="inlineStr"/>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>Cross-border payments platform powering merchant payments, payouts, and remittances across Africa and other emerging markets</t>
+          <t>AI-native Medicare navigation platform pairing licensed advisors with software to help seniors choose and manage Medicare plans</t>
         </is>
       </c>
       <c r="K6" s="3" t="inlineStr">
@@ -1033,28 +1033,28 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>15-Jun-26</t>
+          <t>16-Jun-26</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Interchecks</t>
+          <t>Flutterwave</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Bettor Capital</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="n">
-        <v>50</v>
-      </c>
-      <c r="G7" s="2" t="inlineStr"/>
+          <t>Ripple (strategic)</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr"/>
+      <c r="G7" s="2" t="n">
+        <v>3200</v>
+      </c>
       <c r="H7" s="2" t="inlineStr"/>
       <c r="I7" s="2" t="inlineStr"/>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>Instant payments and money-movement infrastructure serving sportsbooks, fintechs, and financial institutions through a single API</t>
+          <t>Cross-border payments platform powering merchant payments, payouts, and remittances across Africa and other emerging markets</t>
         </is>
       </c>
       <c r="K7" s="3" t="inlineStr">
@@ -1071,22 +1071,22 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>17-Jun-26</t>
+          <t>15-Jun-26</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>BIPO</t>
+          <t>Interchecks</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Apis Partners</t>
+          <t>Bettor Capital</t>
         </is>
       </c>
       <c r="F8" s="2" t="n">
@@ -1097,7 +1097,7 @@
       <c r="I8" s="2" t="inlineStr"/>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Payroll-payments and embedded workforce-finance platform offering global payroll, HR management, and employer-of-record services across 170+ markets</t>
+          <t>Instant payments and money-movement infrastructure serving sportsbooks, fintechs, and financial institutions through a single API</t>
         </is>
       </c>
       <c r="K8" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Add D360 Bank (Saudi digital bank, $400M) to week-ending-2026-06-19 raises
</commit_message>
<xml_diff>
--- a/Weekly_Fintech_Deals_2026-06-19.xlsx
+++ b/Weekly_Fintech_Deals_2026-06-19.xlsx
@@ -12,7 +12,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'M&amp;A'!$A$1:$K$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Growth Capital Raises'!$A$1:$K$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Growth Capital Raises'!$A$1:$K$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -732,7 +732,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K9"/>
+  <dimension ref="A1:K10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -851,38 +851,40 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Capital Markets Tech</t>
+          <t>Banking &amp; Lending Tech</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Saudi Arabia</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>16-Jun-26</t>
+          <t>14-Jun-26</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Chronograph</t>
+          <t>D360 Bank</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Sixth Street Growth</t>
+          <t>Public Investment Fund, Derayah Financial</t>
         </is>
       </c>
       <c r="F3" s="2" t="n">
-        <v>140</v>
-      </c>
-      <c r="G3" s="2" t="inlineStr"/>
+        <v>400</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>1600</v>
+      </c>
       <c r="H3" s="2" t="inlineStr"/>
       <c r="I3" s="2" t="inlineStr"/>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Portfolio monitoring, reporting, and diligence software for private capital investors across private equity and private credit</t>
+          <t>Saudi Arabia's first licensed digital bank, providing consumer and SME financing, deposits, and API-banking services to over three million customers</t>
         </is>
       </c>
       <c r="K3" s="3" t="inlineStr">
@@ -894,38 +896,38 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Corporate Financial Function</t>
+          <t>Capital Markets Tech</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>17-Jun-26</t>
+          <t>16-Jun-26</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>BIPO</t>
+          <t>Chronograph</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Apis Partners</t>
+          <t>Sixth Street Growth</t>
         </is>
       </c>
       <c r="F4" s="2" t="n">
-        <v>50</v>
+        <v>140</v>
       </c>
       <c r="G4" s="2" t="inlineStr"/>
       <c r="H4" s="2" t="inlineStr"/>
       <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>Payroll-payments and embedded workforce-finance platform offering global payroll, HR management, and employer-of-record services across 170+ markets</t>
+          <t>Portfolio monitoring, reporting, and diligence software for private capital investors across private equity and private credit</t>
         </is>
       </c>
       <c r="K4" s="3" t="inlineStr">
@@ -937,12 +939,12 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Financial Info &amp; Analytics</t>
+          <t>Corporate Financial Function</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Singapore</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -952,23 +954,23 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Behavox</t>
+          <t>BIPO</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>HPS Investment Partners</t>
+          <t>Apis Partners</t>
         </is>
       </c>
       <c r="F5" s="2" t="n">
-        <v>175</v>
+        <v>50</v>
       </c>
       <c r="G5" s="2" t="inlineStr"/>
       <c r="H5" s="2" t="inlineStr"/>
       <c r="I5" s="2" t="inlineStr"/>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>AI-native compliance and risk platform that unifies communications surveillance and controls for banks, asset managers, and other regulated institutions</t>
+          <t>Payroll-payments and embedded workforce-finance platform offering global payroll, HR management, and employer-of-record services across 170+ markets</t>
         </is>
       </c>
       <c r="K5" s="3" t="inlineStr">
@@ -980,7 +982,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>InsurTech</t>
+          <t>Financial Info &amp; Analytics</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -990,28 +992,28 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>18-Jun-26</t>
+          <t>17-Jun-26</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Connie Health</t>
+          <t>Behavox</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>HealthQuest Capital</t>
+          <t>HPS Investment Partners</t>
         </is>
       </c>
       <c r="F6" s="2" t="n">
-        <v>40</v>
+        <v>175</v>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
       <c r="H6" s="2" t="inlineStr"/>
       <c r="I6" s="2" t="inlineStr"/>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>AI-native Medicare navigation platform pairing licensed advisors with software to help seniors choose and manage Medicare plans</t>
+          <t>AI-native compliance and risk platform that unifies communications surveillance and controls for banks, asset managers, and other regulated institutions</t>
         </is>
       </c>
       <c r="K6" s="3" t="inlineStr">
@@ -1023,7 +1025,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Payments</t>
+          <t>InsurTech</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -1033,28 +1035,28 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>16-Jun-26</t>
+          <t>18-Jun-26</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Flutterwave</t>
+          <t>Connie Health</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Ripple (strategic)</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr"/>
-      <c r="G7" s="2" t="n">
-        <v>3200</v>
-      </c>
+          <t>HealthQuest Capital</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="G7" s="2" t="inlineStr"/>
       <c r="H7" s="2" t="inlineStr"/>
       <c r="I7" s="2" t="inlineStr"/>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>Cross-border payments platform powering merchant payments, payouts, and remittances across Africa and other emerging markets</t>
+          <t>AI-native Medicare navigation platform pairing licensed advisors with software to help seniors choose and manage Medicare plans</t>
         </is>
       </c>
       <c r="K7" s="3" t="inlineStr">
@@ -1076,28 +1078,28 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>15-Jun-26</t>
+          <t>16-Jun-26</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Interchecks</t>
+          <t>Flutterwave</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Bettor Capital</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="n">
-        <v>50</v>
-      </c>
-      <c r="G8" s="2" t="inlineStr"/>
+          <t>Ripple (strategic)</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr"/>
+      <c r="G8" s="2" t="n">
+        <v>3200</v>
+      </c>
       <c r="H8" s="2" t="inlineStr"/>
       <c r="I8" s="2" t="inlineStr"/>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Instant payments and money-movement infrastructure serving sportsbooks, fintechs, and financial institutions through a single API</t>
+          <t>Cross-border payments platform powering merchant payments, payouts, and remittances across Africa and other emerging markets</t>
         </is>
       </c>
       <c r="K8" s="3" t="inlineStr">
@@ -1119,38 +1121,81 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>17-Jun-26</t>
+          <t>15-Jun-26</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Trace Finance</t>
+          <t>Interchecks</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>CoinFund</t>
+          <t>Bettor Capital</t>
         </is>
       </c>
       <c r="F9" s="2" t="n">
-        <v>32</v>
+        <v>50</v>
       </c>
       <c r="G9" s="2" t="inlineStr"/>
       <c r="H9" s="2" t="inlineStr"/>
       <c r="I9" s="2" t="inlineStr"/>
       <c r="J9" s="2" t="inlineStr">
         <is>
+          <t>Instant payments and money-movement infrastructure serving sportsbooks, fintechs, and financial institutions through a single API</t>
+        </is>
+      </c>
+      <c r="K9" s="3" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Payments</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>17-Jun-26</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Trace Finance</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>CoinFund</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="G10" s="2" t="inlineStr"/>
+      <c r="H10" s="2" t="inlineStr"/>
+      <c r="I10" s="2" t="inlineStr"/>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
           <t>Regulated cross-border banking and stablecoin-settlement infrastructure connecting the US, Brazil, and other emerging markets</t>
         </is>
       </c>
-      <c r="K9" s="3" t="inlineStr">
+      <c r="K10" s="3" t="inlineStr">
         <is>
           <t>Link</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K9"/>
+  <autoFilter ref="A1:K10"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K3" r:id="rId2"/>
@@ -1160,6 +1205,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K7" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K8" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K10" r:id="rId9"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Festina Finance (Asset & Wealth Tech) - now 8/8 sectors for week-ending-2026-06-19
</commit_message>
<xml_diff>
--- a/Weekly_Fintech_Deals_2026-06-19.xlsx
+++ b/Weekly_Fintech_Deals_2026-06-19.xlsx
@@ -12,7 +12,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'M&amp;A'!$A$1:$K$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Growth Capital Raises'!$A$1:$K$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Growth Capital Raises'!$A$1:$K$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -732,7 +732,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K10"/>
+  <dimension ref="A1:K11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -808,38 +808,40 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Banking &amp; Lending Tech</t>
+          <t>Asset &amp; Wealth Tech</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Denmark</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>17-Jun-26</t>
+          <t>19-Jun-26</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Karta</t>
+          <t>Festina Finance</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Galaxy Ventures, Community Investment Management</t>
+          <t>Birchway Capital</t>
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>140</v>
-      </c>
-      <c r="G2" s="2" t="inlineStr"/>
+        <v>27</v>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>216</v>
+      </c>
       <c r="H2" s="2" t="inlineStr"/>
       <c r="I2" s="2" t="inlineStr"/>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>Provider of WhatsApp-run US credit cards for credit-invisible international travelers and non-residents, distributed through private banks and wealth managers</t>
+          <t>Cloud-native, modular system-of-record platform for pensions, life insurance, and financial planning used by pension funds, insurers, banks, and wealth managers across Europe</t>
         </is>
       </c>
       <c r="K2" s="3" t="inlineStr">
@@ -856,35 +858,33 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Saudi Arabia</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>14-Jun-26</t>
+          <t>17-Jun-26</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>D360 Bank</t>
+          <t>Karta</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Public Investment Fund, Derayah Financial</t>
+          <t>Galaxy Ventures, Community Investment Management</t>
         </is>
       </c>
       <c r="F3" s="2" t="n">
-        <v>400</v>
-      </c>
-      <c r="G3" s="2" t="n">
-        <v>1600</v>
-      </c>
+        <v>140</v>
+      </c>
+      <c r="G3" s="2" t="inlineStr"/>
       <c r="H3" s="2" t="inlineStr"/>
       <c r="I3" s="2" t="inlineStr"/>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Saudi Arabia's first licensed digital bank, providing consumer and SME financing, deposits, and API-banking services to over three million customers</t>
+          <t>Provider of WhatsApp-run US credit cards for credit-invisible international travelers and non-residents, distributed through private banks and wealth managers</t>
         </is>
       </c>
       <c r="K3" s="3" t="inlineStr">
@@ -896,38 +896,40 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Capital Markets Tech</t>
+          <t>Banking &amp; Lending Tech</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Saudi Arabia</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>16-Jun-26</t>
+          <t>14-Jun-26</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Chronograph</t>
+          <t>D360 Bank</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Sixth Street Growth</t>
+          <t>Public Investment Fund, Derayah Financial</t>
         </is>
       </c>
       <c r="F4" s="2" t="n">
-        <v>140</v>
-      </c>
-      <c r="G4" s="2" t="inlineStr"/>
+        <v>400</v>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>1600</v>
+      </c>
       <c r="H4" s="2" t="inlineStr"/>
       <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>Portfolio monitoring, reporting, and diligence software for private capital investors across private equity and private credit</t>
+          <t>Saudi Arabia's first licensed digital bank, providing consumer and SME financing, deposits, and API-banking services to over three million customers</t>
         </is>
       </c>
       <c r="K4" s="3" t="inlineStr">
@@ -939,38 +941,38 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Corporate Financial Function</t>
+          <t>Capital Markets Tech</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>17-Jun-26</t>
+          <t>16-Jun-26</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>BIPO</t>
+          <t>Chronograph</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Apis Partners</t>
+          <t>Sixth Street Growth</t>
         </is>
       </c>
       <c r="F5" s="2" t="n">
-        <v>50</v>
+        <v>140</v>
       </c>
       <c r="G5" s="2" t="inlineStr"/>
       <c r="H5" s="2" t="inlineStr"/>
       <c r="I5" s="2" t="inlineStr"/>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Payroll-payments and embedded workforce-finance platform offering global payroll, HR management, and employer-of-record services across 170+ markets</t>
+          <t>Portfolio monitoring, reporting, and diligence software for private capital investors across private equity and private credit</t>
         </is>
       </c>
       <c r="K5" s="3" t="inlineStr">
@@ -982,12 +984,12 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Financial Info &amp; Analytics</t>
+          <t>Corporate Financial Function</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Singapore</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -997,23 +999,23 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Behavox</t>
+          <t>BIPO</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>HPS Investment Partners</t>
+          <t>Apis Partners</t>
         </is>
       </c>
       <c r="F6" s="2" t="n">
-        <v>175</v>
+        <v>50</v>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
       <c r="H6" s="2" t="inlineStr"/>
       <c r="I6" s="2" t="inlineStr"/>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>AI-native compliance and risk platform that unifies communications surveillance and controls for banks, asset managers, and other regulated institutions</t>
+          <t>Payroll-payments and embedded workforce-finance platform offering global payroll, HR management, and employer-of-record services across 170+ markets</t>
         </is>
       </c>
       <c r="K6" s="3" t="inlineStr">
@@ -1025,7 +1027,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>InsurTech</t>
+          <t>Financial Info &amp; Analytics</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -1035,28 +1037,28 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>18-Jun-26</t>
+          <t>17-Jun-26</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Connie Health</t>
+          <t>Behavox</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>HealthQuest Capital</t>
+          <t>HPS Investment Partners</t>
         </is>
       </c>
       <c r="F7" s="2" t="n">
-        <v>40</v>
+        <v>175</v>
       </c>
       <c r="G7" s="2" t="inlineStr"/>
       <c r="H7" s="2" t="inlineStr"/>
       <c r="I7" s="2" t="inlineStr"/>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>AI-native Medicare navigation platform pairing licensed advisors with software to help seniors choose and manage Medicare plans</t>
+          <t>AI-native compliance and risk platform that unifies communications surveillance and controls for banks, asset managers, and other regulated institutions</t>
         </is>
       </c>
       <c r="K7" s="3" t="inlineStr">
@@ -1068,7 +1070,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Payments</t>
+          <t>InsurTech</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -1078,28 +1080,28 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>16-Jun-26</t>
+          <t>18-Jun-26</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Flutterwave</t>
+          <t>Connie Health</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Ripple (strategic)</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr"/>
-      <c r="G8" s="2" t="n">
-        <v>3200</v>
-      </c>
+          <t>HealthQuest Capital</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="G8" s="2" t="inlineStr"/>
       <c r="H8" s="2" t="inlineStr"/>
       <c r="I8" s="2" t="inlineStr"/>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Cross-border payments platform powering merchant payments, payouts, and remittances across Africa and other emerging markets</t>
+          <t>AI-native Medicare navigation platform pairing licensed advisors with software to help seniors choose and manage Medicare plans</t>
         </is>
       </c>
       <c r="K8" s="3" t="inlineStr">
@@ -1121,28 +1123,28 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>15-Jun-26</t>
+          <t>16-Jun-26</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Interchecks</t>
+          <t>Flutterwave</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Bettor Capital</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="n">
-        <v>50</v>
-      </c>
-      <c r="G9" s="2" t="inlineStr"/>
+          <t>Ripple (strategic)</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr"/>
+      <c r="G9" s="2" t="n">
+        <v>3200</v>
+      </c>
       <c r="H9" s="2" t="inlineStr"/>
       <c r="I9" s="2" t="inlineStr"/>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>Instant payments and money-movement infrastructure serving sportsbooks, fintechs, and financial institutions through a single API</t>
+          <t>Cross-border payments platform powering merchant payments, payouts, and remittances across Africa and other emerging markets</t>
         </is>
       </c>
       <c r="K9" s="3" t="inlineStr">
@@ -1164,38 +1166,81 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>17-Jun-26</t>
+          <t>15-Jun-26</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Trace Finance</t>
+          <t>Interchecks</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>CoinFund</t>
+          <t>Bettor Capital</t>
         </is>
       </c>
       <c r="F10" s="2" t="n">
-        <v>32</v>
+        <v>50</v>
       </c>
       <c r="G10" s="2" t="inlineStr"/>
       <c r="H10" s="2" t="inlineStr"/>
       <c r="I10" s="2" t="inlineStr"/>
       <c r="J10" s="2" t="inlineStr">
         <is>
+          <t>Instant payments and money-movement infrastructure serving sportsbooks, fintechs, and financial institutions through a single API</t>
+        </is>
+      </c>
+      <c r="K10" s="3" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Payments</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>17-Jun-26</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Trace Finance</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>CoinFund</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="G11" s="2" t="inlineStr"/>
+      <c r="H11" s="2" t="inlineStr"/>
+      <c r="I11" s="2" t="inlineStr"/>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
           <t>Regulated cross-border banking and stablecoin-settlement infrastructure connecting the US, Brazil, and other emerging markets</t>
         </is>
       </c>
-      <c r="K10" s="3" t="inlineStr">
+      <c r="K11" s="3" t="inlineStr">
         <is>
           <t>Link</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K10"/>
+  <autoFilter ref="A1:K11"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K3" r:id="rId2"/>
@@ -1206,6 +1251,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K8" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K9" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K11" r:id="rId10"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>